<commit_message>
fix merged cells bug + 15 strategies engine verified exit 0
</commit_message>
<xml_diff>
--- a/trading/paper_trading/paper_trading.xlsx
+++ b/trading/paper_trading/paper_trading.xlsx
@@ -571,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -629,7 +629,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Supertrend (10,3)</t>
+          <t>Supertrend (10,3) + EMA50</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -653,6 +653,7 @@
       <c r="H2" s="2" t="n">
         <v>0</v>
       </c>
+      <c r="I2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -681,6 +682,7 @@
       <c r="H3" s="2" t="n">
         <v>0</v>
       </c>
+      <c r="I3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -709,6 +711,7 @@
       <c r="H4" s="2" t="n">
         <v>0</v>
       </c>
+      <c r="I4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -737,6 +740,7 @@
       <c r="H5" s="2" t="n">
         <v>0</v>
       </c>
+      <c r="I5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -765,6 +769,297 @@
       <c r="H6" s="2" t="n">
         <v>0</v>
       </c>
+      <c r="I6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>EMA + ADX Trend</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>SMA 50/200 Cross</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Donchian 20 Breakout</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Triple EMA (9/21/50)</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Keltner Breakout</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Volume Surge Momentum</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>MACD Histogram Flip</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>ATR Breakout</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Hull MA + RSI</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Price Structure Break</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -777,7 +1072,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -793,9 +1088,6 @@
           <t>PAPER TRADING ACCOUNT</t>
         </is>
       </c>
-      <c r="B1" s="7" t="n"/>
-      <c r="C1" s="7" t="n"/>
-      <c r="D1" s="8" t="n"/>
       <c r="E1" s="1" t="n"/>
     </row>
     <row r="3">
@@ -841,7 +1133,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -854,12 +1146,29 @@
         <v>0</v>
       </c>
     </row>
+    <row r="8">
+      <c r="B8" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+    </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
           <t>MONTHLY P&amp;L</t>
         </is>
       </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>0.0:1</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -915,11 +1224,72 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>₹100,000</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>₹100,000</t>
+        </is>
+      </c>
+      <c r="D60" s="10" t="inlineStr">
+        <is>
+          <t>₹+0</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>₹+0</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A10:D10"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
v2: 15 strategies independent per-stock positions
</commit_message>
<xml_diff>
--- a/trading/paper_trading/paper_trading.xlsx
+++ b/trading/paper_trading/paper_trading.xlsx
@@ -49,7 +49,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -65,6 +65,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -114,7 +119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -128,6 +133,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -493,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -557,6 +564,48 @@
       <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>11155</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>10996</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G2" s="11" t="n">
+        <v>-318</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>VWAP Pullback</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Exit by VWAP Pullback</t>
         </is>
       </c>
     </row>
@@ -749,19 +798,19 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C6" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="6" t="n">
-        <v>0</v>
+      <c r="F6" s="11" t="n">
+        <v>-318</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>0</v>
@@ -1072,7 +1121,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E60"/>
+  <dimension ref="A1:E79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1110,7 +1159,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹100,000</t>
+          <t>₹99,682</t>
         </is>
       </c>
     </row>
@@ -1120,9 +1169,9 @@
           <t>Total P&amp;L</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>₹+0</t>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>₹-318</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1182,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -1143,18 +1192,18 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.0%</t>
         </is>
       </c>
     </row>
@@ -1289,6 +1338,519 @@
         </is>
       </c>
     </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>₹100,000</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>₹100,000</t>
+        </is>
+      </c>
+      <c r="D61" s="10" t="inlineStr">
+        <is>
+          <t>₹+0</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>₹+0</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>₹100,000</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>₹100,000</t>
+        </is>
+      </c>
+      <c r="D62" s="10" t="inlineStr">
+        <is>
+          <t>₹+0</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>₹+0</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>₹100,000</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>₹100,000</t>
+        </is>
+      </c>
+      <c r="D63" s="10" t="inlineStr">
+        <is>
+          <t>₹+0</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>₹+0</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>₹99,682</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>₹99,682</t>
+        </is>
+      </c>
+      <c r="D64" s="10" t="inlineStr">
+        <is>
+          <t>₹+0</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>₹-318</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>₹99,682</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>₹99,682</t>
+        </is>
+      </c>
+      <c r="D65" s="10" t="inlineStr">
+        <is>
+          <t>₹+0</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>₹-318</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>₹99,682</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>₹99,682</t>
+        </is>
+      </c>
+      <c r="D66" s="10" t="inlineStr">
+        <is>
+          <t>₹+0</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>₹-318</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>₹99,682</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>₹99,682</t>
+        </is>
+      </c>
+      <c r="D67" s="10" t="inlineStr">
+        <is>
+          <t>₹+0</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>₹-318</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>₹99,682</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>₹99,682</t>
+        </is>
+      </c>
+      <c r="D68" s="10" t="inlineStr">
+        <is>
+          <t>₹+0</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>₹-318</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>₹99,682</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>₹99,682</t>
+        </is>
+      </c>
+      <c r="D69" s="10" t="inlineStr">
+        <is>
+          <t>₹+0</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>₹-318</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>₹99,682</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>₹99,682</t>
+        </is>
+      </c>
+      <c r="D70" s="10" t="inlineStr">
+        <is>
+          <t>₹+0</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>₹-318</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>₹99,682</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>₹99,682</t>
+        </is>
+      </c>
+      <c r="D71" s="10" t="inlineStr">
+        <is>
+          <t>₹+0</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>₹-318</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>₹99,682</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>₹99,682</t>
+        </is>
+      </c>
+      <c r="D72" s="10" t="inlineStr">
+        <is>
+          <t>₹+0</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>₹-318</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>₹99,682</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>₹99,682</t>
+        </is>
+      </c>
+      <c r="D73" s="10" t="inlineStr">
+        <is>
+          <t>₹+0</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>₹-318</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>₹99,682</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>₹99,682</t>
+        </is>
+      </c>
+      <c r="D74" s="10" t="inlineStr">
+        <is>
+          <t>₹+0</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>₹-318</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>₹99,682</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>₹99,682</t>
+        </is>
+      </c>
+      <c r="D75" s="10" t="inlineStr">
+        <is>
+          <t>₹+0</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>₹-318</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>₹99,682</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>₹99,682</t>
+        </is>
+      </c>
+      <c r="D76" s="10" t="inlineStr">
+        <is>
+          <t>₹+0</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>₹-318</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>₹99,682</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>₹99,682</t>
+        </is>
+      </c>
+      <c r="D77" s="10" t="inlineStr">
+        <is>
+          <t>₹+0</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>₹-318</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>₹99,682</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>₹99,682</t>
+        </is>
+      </c>
+      <c r="D78" s="10" t="inlineStr">
+        <is>
+          <t>₹+0</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>₹-318</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>₹99,682</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>₹99,682</t>
+        </is>
+      </c>
+      <c r="D79" s="10" t="inlineStr">
+        <is>
+          <t>₹+0</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>₹-318</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
v3: 50 stocks, 15min intraday, auto SL/TP, 10min cron
</commit_message>
<xml_diff>
--- a/trading/paper_trading/paper_trading.xlsx
+++ b/trading/paper_trading/paper_trading.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,6 +47,14 @@
       <b val="1"/>
       <color rgb="004472C4"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="5">
@@ -119,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -135,6 +143,11 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -678,7 +691,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Supertrend (10,3) + EMA50</t>
+          <t>Supertrend+EMA50</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -699,15 +712,21 @@
       <c r="G2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>₹6,666</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>EMA Crossover (6/30)</t>
+          <t>EMA Cross 6/30</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
@@ -728,15 +747,21 @@
       <c r="G3" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>₹6,666</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>RSI + MACD</t>
+          <t>RSI+MACD</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -757,10 +782,16 @@
       <c r="G4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>₹6,666</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -786,10 +817,16 @@
       <c r="G5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>₹6,666</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -798,32 +835,38 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C6" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E6" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="11" t="n">
-        <v>-318</v>
+      <c r="F6" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>₹6,666</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>EMA + ADX Trend</t>
+          <t>EMA+ADX Trend</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
@@ -844,10 +887,16 @@
       <c r="G7" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>₹6,666</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -873,15 +922,21 @@
       <c r="G8" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>₹6,666</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Donchian 20 Breakout</t>
+          <t>Donchian 20</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
@@ -902,15 +957,21 @@
       <c r="G9" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>₹6,666</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Triple EMA (9/21/50)</t>
+          <t>Triple EMA 9/21/50</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -931,10 +992,16 @@
       <c r="G10" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>₹6,666</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -960,15 +1027,21 @@
       <c r="G11" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H11" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>₹6,666</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Volume Surge Momentum</t>
+          <t>Vol Surge</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -989,15 +1062,21 @@
       <c r="G12" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>₹6,666</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>MACD Histogram Flip</t>
+          <t>MACD Hist Flip</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
@@ -1018,10 +1097,16 @@
       <c r="G13" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>₹6,666</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1047,15 +1132,21 @@
       <c r="G14" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>₹6,666</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Hull MA + RSI</t>
+          <t>Hull MA+RSI</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
@@ -1076,15 +1167,21 @@
       <c r="G15" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H15" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="2" t="inlineStr"/>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>₹6,666</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Price Structure Break</t>
+          <t>Price Structure</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1105,10 +1202,16 @@
       <c r="G16" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H16" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>₹6,666</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1132,47 +1235,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>PAPER TRADING ACCOUNT</t>
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>ACCOUNT OVERVIEW</t>
         </is>
       </c>
       <c r="E1" s="1" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>Start Capital</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>₹100,000</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Starting Capital</t>
+          <t>Current Capital</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>₹1,00,000</t>
+          <t>₹99,990</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Current Balance</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>₹99,682</t>
+          <t>Total P&amp;L</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>₹-10</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Total P&amp;L</t>
-        </is>
-      </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>₹-318</t>
-        </is>
+          <t>Total Trades</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -1182,17 +1295,19 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Total Closed Trades</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="n">
-        <v>1</v>
+          <t>Return %</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>-0.01%</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -1201,6 +1316,11 @@
       </c>
     </row>
     <row r="9">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>PER-STRATEGY CAPITAL</t>
+        </is>
+      </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
           <t>0.0%</t>
@@ -1210,24 +1330,24 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>MONTHLY P&amp;L</t>
+          <t>Supertrend+EMA50</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>0.0:1</t>
+          <t>₹6,666</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Month</t>
+          <t>EMA Cross 6/30</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Starting Balance</t>
+          <t>₹6,666</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1249,12 +1369,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Sep 2026</t>
+          <t>RSI+MACD</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>₹1,00,000</t>
+          <t>₹6,666</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1273,44 +1393,150 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>BB Squeeze</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>₹6,666</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>VWAP Pullback</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>₹6,666</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>EMA+ADX Trend</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>₹6,666</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SMA 50/200 Cross</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>₹6,666</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Donchian 20</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>₹6,666</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Triple EMA 9/21/50</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>₹6,666</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Keltner Breakout</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>₹6,666</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Vol Surge</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>₹6,666</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>MACD Hist Flip</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>₹6,666</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>ATR Breakout</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>₹6,666</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Hull MA+RSI</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>₹6,666</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Price Structure</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>₹6,666</t>
+        </is>
+      </c>
+    </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix Supertrend bug: was using Close for band width instead of ATR
</commit_message>
<xml_diff>
--- a/trading/paper_trading/paper_trading.xlsx
+++ b/trading/paper_trading/paper_trading.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,16 +38,25 @@
       <b val="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -55,15 +64,24 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -495,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -542,6 +560,1756 @@
       <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Return%</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>S7/2</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>S10/2</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>S10/3</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>S14/3</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>S20/4</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>E5/13</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>E6/30</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>E8/21</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>E10/50</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>E20/50</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>RSI30</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>RSI25</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>RSI75</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>RSIDiv</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>MHist</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>MACross</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>MACDV</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>BBSqz</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>BB%&lt;.2</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I20" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>BB%&gt;.8</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>BBNar</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>BBExt</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>ADX25</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>ADX30</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>ADX20</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I26" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>D20</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>D10</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I28" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>D55</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I29" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>VSurge</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I30" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>VClimax</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I31" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>VAccum</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I32" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>VDist</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>KBreak</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I34" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>KCTouch</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I35" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>KReject</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I36" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>StrBreak</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I37" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>InBar</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I38" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Engulf</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I39" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>3Bar</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I40" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>ATR1.5</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I41" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>ATR2</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I42" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>ATRAve</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I43" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>H9/18</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I44" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>H9/50</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I45" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>VWAPPull</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I46" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>VWAPDiv</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D47" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I47" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>ROCS</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D48" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I48" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>ROCV</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D49" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I49" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>PRIROC</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D50" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I50" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Confluence</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D51" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F51" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H51" s="4" t="inlineStr">
+        <is>
+          <t>₹10,000</t>
+        </is>
+      </c>
+      <c r="I51" s="4" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
         </is>
       </c>
     </row>
@@ -556,7 +2324,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -572,7 +2340,7 @@
           <t>Start</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>₹500,000</t>
         </is>
@@ -584,7 +2352,7 @@
           <t>Capital</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>₹500,000</t>
         </is>
@@ -596,9 +2364,9 @@
           <t>P&amp;L</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>₹0</t>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>₹+0</t>
         </is>
       </c>
     </row>
@@ -608,7 +2376,7 @@
           <t>Trades</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -618,8 +2386,8 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>0</v>
+      <c r="B6" s="4" t="n">
+        <v>346</v>
       </c>
     </row>
     <row r="7">
@@ -628,16 +2396,59 @@
           <t>Return</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>+0.00%</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>50 STRATS | 100 STOCKS | SL 1.5x TP 3x | 10MIN</t>
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>🧠 PSYCHOLOGY RULES</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Max 2% risk/trade ✓ | Max 5 pos ✓ | Trend filter ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Cool-off 3 losses ✓ | Half-size on 10% DD ✓ | No avg-down ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>DD%</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Loss streak</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>50 STRATS | 100 STOCKS | SL 1.5x TP 3.0x | 10MIN</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: news once per hour + remove default Excel Sheet tab
</commit_message>
<xml_diff>
--- a/trading/paper_trading/paper_trading.xlsx
+++ b/trading/paper_trading/paper_trading.xlsx
@@ -43,7 +43,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -53,6 +53,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -74,7 +79,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -82,6 +87,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -447,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -499,6 +505,1018 @@
       <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Exit Reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>14:21</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>AAVAS</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>PRIROC</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="n">
+        <v>1262</v>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>1261.3</v>
+      </c>
+      <c r="H2" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I2" s="7" t="n">
+        <v>-1</v>
+      </c>
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>SIG</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>14:21</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>COCHINSHIP</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>PRIROC</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>COVER</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>1292.9</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>1297.2</v>
+      </c>
+      <c r="H3" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I3" s="7" t="n">
+        <v>-9</v>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>SIG</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>14:21</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>GODREJIND</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>RSI75</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>COVER</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>1063.4</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>1063.6</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>SIG</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>14:21</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>JASH</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>ADX30</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>595.25</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>596</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I5" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>SIG</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>14:21</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>JYOTIRES</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>E20/50</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>850</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>842.92</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I6" s="7" t="n">
+        <v>-21</v>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>14:21</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>JYOTIRES</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>ADX25</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>850</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>842.92</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I7" s="7" t="n">
+        <v>-21</v>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>14:21</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>JYOTIRES</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>ADX20</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>850</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>842.92</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I8" s="7" t="n">
+        <v>-21</v>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>14:21</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>JYOTIRES</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>D10</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>850</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>842.92</v>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I9" s="7" t="n">
+        <v>-21</v>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>14:21</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>JYOTIRES</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>VAccum</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>850</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>842.92</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I10" s="7" t="n">
+        <v>-21</v>
+      </c>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>14:21</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>JYOTIRES</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>StrBreak</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>850</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>842.92</v>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I11" s="7" t="n">
+        <v>-21</v>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>14:21</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>JYOTIRES</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>ATR1.5</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>850</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>842.92</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I12" s="7" t="n">
+        <v>-21</v>
+      </c>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>14:21</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>JYOTIRES</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>H9/18</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>850</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>842.92</v>
+      </c>
+      <c r="H13" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I13" s="7" t="n">
+        <v>-21</v>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>14:21</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>JYOTIRES</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>H9/50</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>850</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>842.92</v>
+      </c>
+      <c r="H14" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I14" s="7" t="n">
+        <v>-21</v>
+      </c>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>14:21</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>JYOTIRES</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>VWAPPull</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>850</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>842.92</v>
+      </c>
+      <c r="H15" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I15" s="7" t="n">
+        <v>-21</v>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>14:21</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>JYOTIRES</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>PRIROC</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>850</v>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>842.92</v>
+      </c>
+      <c r="H16" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I16" s="7" t="n">
+        <v>-21</v>
+      </c>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>14:21</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>JYOTIRES</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Confluence</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>850</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>842.92</v>
+      </c>
+      <c r="H17" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I17" s="7" t="n">
+        <v>-21</v>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>14:21</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>KPRMILL</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>BBNar</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>COVER</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>1094.8</v>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>1097</v>
+      </c>
+      <c r="H18" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I18" s="7" t="n">
+        <v>-4</v>
+      </c>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>SIG</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>14:21</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>KSCL</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>BBNar</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>COVER</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>744</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>746.85</v>
+      </c>
+      <c r="H19" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I19" s="7" t="n">
+        <v>-11</v>
+      </c>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>SIG</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>14:21</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>MARICO</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Engulf</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>COVER</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>800.65</v>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>801.3</v>
+      </c>
+      <c r="H20" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I20" s="7" t="n">
+        <v>-2</v>
+      </c>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>SIG</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>14:21</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>MAYURUNIQ</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>BBNar</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>731.1</v>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>730.3</v>
+      </c>
+      <c r="H21" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I21" s="7" t="n">
+        <v>-3</v>
+      </c>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>SIG</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>14:21</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>MAYURUNIQ</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>ADX30</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>731.1</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>730.3</v>
+      </c>
+      <c r="H22" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I22" s="7" t="n">
+        <v>-3</v>
+      </c>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>SIG</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>14:21</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>RELIANCE</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>BBNar</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>COVER</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>1190.5</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>1191</v>
+      </c>
+      <c r="H23" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I23" s="7" t="n">
+        <v>-1</v>
+      </c>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>SIG</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>14:21</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>WHIRLPOOL</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>PRIROC</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>894.95</v>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>893.45</v>
+      </c>
+      <c r="H24" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I24" s="7" t="n">
+        <v>-4</v>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>SIG</t>
         </is>
       </c>
     </row>
@@ -885,31 +1903,31 @@
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C11" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E11" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F11" s="5" t="n">
-        <v>0</v>
+      <c r="F11" s="7" t="n">
+        <v>-21</v>
       </c>
       <c r="G11" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>₹10,000</t>
+          <t>₹9,958</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>+0.0%</t>
+          <t>-0.4%</t>
         </is>
       </c>
     </row>
@@ -990,16 +2008,16 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C14" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D14" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="F14" s="5" t="n">
         <v>0</v>
@@ -1014,7 +2032,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>+0.0%</t>
+          <t>-0.0%</t>
         </is>
       </c>
     </row>
@@ -1270,31 +2288,31 @@
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C22" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E22" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F22" s="5" t="n">
-        <v>0</v>
+      <c r="F22" s="7" t="n">
+        <v>-19</v>
       </c>
       <c r="G22" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>₹10,000</t>
+          <t>₹9,961</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>+0.0%</t>
+          <t>-0.4%</t>
         </is>
       </c>
     </row>
@@ -1340,31 +2358,31 @@
         </is>
       </c>
       <c r="B24" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C24" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E24" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F24" s="5" t="n">
-        <v>0</v>
+      <c r="F24" s="7" t="n">
+        <v>-21</v>
       </c>
       <c r="G24" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>₹10,000</t>
+          <t>₹9,958</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>+0.0%</t>
+          <t>-0.4%</t>
         </is>
       </c>
     </row>
@@ -1375,26 +2393,26 @@
         </is>
       </c>
       <c r="B25" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C25" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F25" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>0</v>
+        <v>1.33</v>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>₹10,000</t>
+          <t>₹10,002</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
@@ -1410,31 +2428,31 @@
         </is>
       </c>
       <c r="B26" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C26" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E26" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F26" s="5" t="n">
-        <v>0</v>
+      <c r="F26" s="7" t="n">
+        <v>-21</v>
       </c>
       <c r="G26" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>₹10,000</t>
+          <t>₹9,958</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>+0.0%</t>
+          <t>-0.4%</t>
         </is>
       </c>
     </row>
@@ -1480,31 +2498,31 @@
         </is>
       </c>
       <c r="B28" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C28" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E28" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F28" s="5" t="n">
-        <v>0</v>
+      <c r="F28" s="7" t="n">
+        <v>-21</v>
       </c>
       <c r="G28" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>₹10,000</t>
+          <t>₹9,958</t>
         </is>
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>+0.0%</t>
+          <t>-0.4%</t>
         </is>
       </c>
     </row>
@@ -1620,31 +2638,31 @@
         </is>
       </c>
       <c r="B32" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C32" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E32" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F32" s="5" t="n">
-        <v>0</v>
+      <c r="F32" s="7" t="n">
+        <v>-21</v>
       </c>
       <c r="G32" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>₹10,000</t>
+          <t>₹9,958</t>
         </is>
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>+0.0%</t>
+          <t>-0.4%</t>
         </is>
       </c>
     </row>
@@ -1795,31 +2813,31 @@
         </is>
       </c>
       <c r="B37" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C37" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E37" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F37" s="5" t="n">
-        <v>0</v>
+      <c r="F37" s="7" t="n">
+        <v>-21</v>
       </c>
       <c r="G37" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>₹10,000</t>
+          <t>₹9,958</t>
         </is>
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>+0.0%</t>
+          <t>-0.4%</t>
         </is>
       </c>
     </row>
@@ -1865,31 +2883,31 @@
         </is>
       </c>
       <c r="B39" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C39" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E39" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F39" s="5" t="n">
-        <v>0</v>
+      <c r="F39" s="7" t="n">
+        <v>-2</v>
       </c>
       <c r="G39" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>₹10,000</t>
+          <t>₹9,996</t>
         </is>
       </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>+0.0%</t>
+          <t>-0.0%</t>
         </is>
       </c>
     </row>
@@ -1935,31 +2953,31 @@
         </is>
       </c>
       <c r="B41" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C41" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E41" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F41" s="5" t="n">
-        <v>0</v>
+      <c r="F41" s="7" t="n">
+        <v>-21</v>
       </c>
       <c r="G41" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>₹10,000</t>
+          <t>₹9,958</t>
         </is>
       </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>+0.0%</t>
+          <t>-0.4%</t>
         </is>
       </c>
     </row>
@@ -2040,31 +3058,31 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C44" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D44" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E44" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F44" s="5" t="n">
-        <v>0</v>
+      <c r="F44" s="7" t="n">
+        <v>-21</v>
       </c>
       <c r="G44" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t>₹10,000</t>
+          <t>₹9,958</t>
         </is>
       </c>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>+0.0%</t>
+          <t>-0.4%</t>
         </is>
       </c>
     </row>
@@ -2075,31 +3093,31 @@
         </is>
       </c>
       <c r="B45" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C45" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D45" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E45" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F45" s="5" t="n">
-        <v>0</v>
+      <c r="F45" s="7" t="n">
+        <v>-21</v>
       </c>
       <c r="G45" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H45" s="4" t="inlineStr">
         <is>
-          <t>₹10,000</t>
+          <t>₹9,958</t>
         </is>
       </c>
       <c r="I45" s="4" t="inlineStr">
         <is>
-          <t>+0.0%</t>
+          <t>-0.4%</t>
         </is>
       </c>
     </row>
@@ -2110,31 +3128,31 @@
         </is>
       </c>
       <c r="B46" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C46" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D46" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E46" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F46" s="5" t="n">
-        <v>0</v>
+      <c r="F46" s="7" t="n">
+        <v>-21</v>
       </c>
       <c r="G46" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H46" s="4" t="inlineStr">
         <is>
-          <t>₹10,000</t>
+          <t>₹9,958</t>
         </is>
       </c>
       <c r="I46" s="4" t="inlineStr">
         <is>
-          <t>+0.0%</t>
+          <t>-0.4%</t>
         </is>
       </c>
     </row>
@@ -2250,31 +3268,31 @@
         </is>
       </c>
       <c r="B50" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C50" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E50" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F50" s="5" t="n">
-        <v>0</v>
+      <c r="F50" s="7" t="n">
+        <v>-35</v>
       </c>
       <c r="G50" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H50" s="4" t="inlineStr">
         <is>
-          <t>₹10,000</t>
+          <t>₹9,929</t>
         </is>
       </c>
       <c r="I50" s="4" t="inlineStr">
         <is>
-          <t>+0.0%</t>
+          <t>-0.7%</t>
         </is>
       </c>
     </row>
@@ -2285,31 +3303,31 @@
         </is>
       </c>
       <c r="B51" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C51" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D51" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E51" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F51" s="5" t="n">
-        <v>0</v>
+      <c r="F51" s="7" t="n">
+        <v>-21</v>
       </c>
       <c r="G51" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H51" s="4" t="inlineStr">
         <is>
-          <t>₹10,000</t>
+          <t>₹9,958</t>
         </is>
       </c>
       <c r="I51" s="4" t="inlineStr">
         <is>
-          <t>+0.0%</t>
+          <t>-0.4%</t>
         </is>
       </c>
     </row>
@@ -2354,7 +3372,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>₹500,000</t>
+          <t>₹499,709</t>
         </is>
       </c>
     </row>
@@ -2364,9 +3382,9 @@
           <t>P&amp;L</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>₹+0</t>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>₹-291.0642002649256</t>
         </is>
       </c>
     </row>
@@ -2377,7 +3395,7 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6">
@@ -2387,7 +3405,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>346</v>
+        <v>458</v>
       </c>
     </row>
     <row r="7">
@@ -2398,7 +3416,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>+0.00%</t>
+          <t>-0.06%</t>
         </is>
       </c>
     </row>
@@ -2442,7 +3460,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
     </row>
     <row r="14">

</xml_diff>